<commit_message>
fr core release 2.2.0
</commit_message>
<xml_diff>
--- a/www/ig/fhir/core/CodeSystem-fr-core-cs-circonstances-sortie.xlsx
+++ b/www/ig/fhir/core/CodeSystem-fr-core-cs-circonstances-sortie.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="71">
   <si>
     <t>Property</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.1.0</t>
+    <t>2.2.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-09-04T10:06:33+02:00</t>
+    <t>2026-03-19T12:11:47+01:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -72,10 +72,10 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>Interop'Santé (http://interopsante.org/)</t>
-  </si>
-  <si>
-    <t>InteropSanté (fhir@interopsante.org(work))</t>
+    <t>Interop'Santé (http://interopsante.org)</t>
+  </si>
+  <si>
+    <t>InteropSanté (fhir@interopsante.org(Work))</t>
   </si>
   <si>
     <t>Jurisdiction</t>
@@ -570,7 +570,9 @@
       <c r="C2" t="s" s="2">
         <v>44</v>
       </c>
-      <c r="D2" s="2"/>
+      <c r="D2" t="s" s="2">
+        <v>44</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
@@ -582,7 +584,9 @@
       <c r="C3" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="D3" s="2"/>
+      <c r="D3" t="s" s="2">
+        <v>46</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
@@ -594,7 +598,9 @@
       <c r="C4" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" t="s" s="2">
+        <v>48</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
@@ -606,7 +612,9 @@
       <c r="C5" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="D5" s="2"/>
+      <c r="D5" t="s" s="2">
+        <v>50</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
@@ -618,7 +626,9 @@
       <c r="C6" t="s" s="2">
         <v>52</v>
       </c>
-      <c r="D6" s="2"/>
+      <c r="D6" t="s" s="2">
+        <v>52</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
@@ -630,7 +640,9 @@
       <c r="C7" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="D7" s="2"/>
+      <c r="D7" t="s" s="2">
+        <v>54</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
@@ -642,7 +654,9 @@
       <c r="C8" t="s" s="2">
         <v>56</v>
       </c>
-      <c r="D8" s="2"/>
+      <c r="D8" t="s" s="2">
+        <v>56</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
@@ -654,7 +668,9 @@
       <c r="C9" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="D9" s="2"/>
+      <c r="D9" t="s" s="2">
+        <v>58</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
@@ -666,7 +682,9 @@
       <c r="C10" t="s" s="2">
         <v>60</v>
       </c>
-      <c r="D10" s="2"/>
+      <c r="D10" t="s" s="2">
+        <v>60</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
@@ -678,7 +696,9 @@
       <c r="C11" t="s" s="2">
         <v>62</v>
       </c>
-      <c r="D11" s="2"/>
+      <c r="D11" t="s" s="2">
+        <v>62</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
@@ -690,7 +710,9 @@
       <c r="C12" t="s" s="2">
         <v>64</v>
       </c>
-      <c r="D12" s="2"/>
+      <c r="D12" t="s" s="2">
+        <v>64</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
@@ -702,7 +724,9 @@
       <c r="C13" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="D13" s="2"/>
+      <c r="D13" t="s" s="2">
+        <v>66</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
@@ -714,7 +738,9 @@
       <c r="C14" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="D14" s="2"/>
+      <c r="D14" t="s" s="2">
+        <v>68</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
@@ -726,7 +752,9 @@
       <c r="C15" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="D15" s="2"/>
+      <c r="D15" t="s" s="2">
+        <v>70</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Revert "fr core release 2.2.0"
This reverts commit 5df350bcdbb6fd75aaf1b254b73f12b5e1cceb97.
</commit_message>
<xml_diff>
--- a/www/ig/fhir/core/CodeSystem-fr-core-cs-circonstances-sortie.xlsx
+++ b/www/ig/fhir/core/CodeSystem-fr-core-cs-circonstances-sortie.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
   <si>
     <t>Property</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.2.0</t>
+    <t>2.1.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-19T12:11:47+01:00</t>
+    <t>2024-09-04T10:06:33+02:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -72,10 +72,10 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>Interop'Santé (http://interopsante.org)</t>
-  </si>
-  <si>
-    <t>InteropSanté (fhir@interopsante.org(Work))</t>
+    <t>Interop'Santé (http://interopsante.org/)</t>
+  </si>
+  <si>
+    <t>InteropSanté (fhir@interopsante.org(work))</t>
   </si>
   <si>
     <t>Jurisdiction</t>
@@ -570,9 +570,7 @@
       <c r="C2" t="s" s="2">
         <v>44</v>
       </c>
-      <c r="D2" t="s" s="2">
-        <v>44</v>
-      </c>
+      <c r="D2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
@@ -584,9 +582,7 @@
       <c r="C3" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="D3" t="s" s="2">
-        <v>46</v>
-      </c>
+      <c r="D3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
@@ -598,9 +594,7 @@
       <c r="C4" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="D4" t="s" s="2">
-        <v>48</v>
-      </c>
+      <c r="D4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
@@ -612,9 +606,7 @@
       <c r="C5" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="D5" t="s" s="2">
-        <v>50</v>
-      </c>
+      <c r="D5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
@@ -626,9 +618,7 @@
       <c r="C6" t="s" s="2">
         <v>52</v>
       </c>
-      <c r="D6" t="s" s="2">
-        <v>52</v>
-      </c>
+      <c r="D6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
@@ -640,9 +630,7 @@
       <c r="C7" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="D7" t="s" s="2">
-        <v>54</v>
-      </c>
+      <c r="D7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
@@ -654,9 +642,7 @@
       <c r="C8" t="s" s="2">
         <v>56</v>
       </c>
-      <c r="D8" t="s" s="2">
-        <v>56</v>
-      </c>
+      <c r="D8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
@@ -668,9 +654,7 @@
       <c r="C9" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="D9" t="s" s="2">
-        <v>58</v>
-      </c>
+      <c r="D9" s="2"/>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
@@ -682,9 +666,7 @@
       <c r="C10" t="s" s="2">
         <v>60</v>
       </c>
-      <c r="D10" t="s" s="2">
-        <v>60</v>
-      </c>
+      <c r="D10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
@@ -696,9 +678,7 @@
       <c r="C11" t="s" s="2">
         <v>62</v>
       </c>
-      <c r="D11" t="s" s="2">
-        <v>62</v>
-      </c>
+      <c r="D11" s="2"/>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
@@ -710,9 +690,7 @@
       <c r="C12" t="s" s="2">
         <v>64</v>
       </c>
-      <c r="D12" t="s" s="2">
-        <v>64</v>
-      </c>
+      <c r="D12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
@@ -724,9 +702,7 @@
       <c r="C13" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="D13" t="s" s="2">
-        <v>66</v>
-      </c>
+      <c r="D13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
@@ -738,9 +714,7 @@
       <c r="C14" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="D14" t="s" s="2">
-        <v>68</v>
-      </c>
+      <c r="D14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
@@ -752,9 +726,7 @@
       <c r="C15" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="D15" t="s" s="2">
-        <v>70</v>
-      </c>
+      <c r="D15" s="2"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>